<commit_message>
corpus: array-classes-3 and more array-classes-2 shapes (#874 r7)
array-classes-2 gains the shapes that pin RPX under an array conversion
(SUMPRODUCT(MAX((...)*B1:B3)), SUMPRODUCT(MAX(LEN(...))), LARGE of an
array) and RA parameters (LOOKUP, INDEX of an array, IRR, TREND,
LINEST, FREQUENCY, bare-reference calls). array-classes-3 has Excel
write the newer functions it can (PERCENTILE.INC and the other twins,
XLOOKUP, XMATCH, FILTER, UNIQUE, SORT, SORTBY, IFS, SWITCH, ...), the
Analysis ToolPak's EDATE and WEEKNUM, and XLLTWICE, a function the test
XLL registers (the arrays section builds it), each as a plain cell,
legacy array and dynamic formula.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/corpus/legacy/arrays/array-classes-2.xlsx
+++ b/corpus/legacy/arrays/array-classes-2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boris\source\workbench\docxy-issue-874\corpus\legacy\arrays\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97A38E55-0DF3-40BD-8E82-623914A5FBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{190A2456-47F0-4AC6-A325-6F8D6CF224DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{D8ECD87B-5495-4AFE-AA82-B55EBECA96FC}"/>
+    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{E2D0729D-E716-41B3-90D6-51C2311357EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Cell" sheetId="1" r:id="rId1"/>
@@ -112,8 +112,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -447,8 +448,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8A7F96D-C957-46B2-BBB6-E0A7650C9E39}">
-  <dimension ref="A1:F37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87904B44-C1AF-433D-B235-B8BC8BE9D7AD}">
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -703,6 +704,78 @@
     <row r="37" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F37">
         <f>VLOOKUP(2,A1:B3,2,0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <f>SUMPRODUCT(MAX((C1:C3="x")*B1:B3))</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F39">
+        <f>SUMPRODUCT(LARGE((A1:A3&gt;1)*B1:B3,{1,2}))</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F40" t="e">
+        <f>SUMPRODUCT(MAX(LEN(C1:C3)))</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="41" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <f>LOOKUP(2,1/(A1:A3&gt;1),B1:B3)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F42">
+        <f>INDEX(B1:B3,MATCH(1,INDEX((A1:A3&gt;1)*(C1:C3="x"),0),0))</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F43" s="1">
+        <f>IRR(A1:A3*1-2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F44">
+        <f>LOOKUP(2,A1:A3,B1:B3)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F45" s="1" t="e">
+        <f>IRR(B1:B3)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="46" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F46">
+        <f>SUM(TREND(B1:B3,A1:A3))</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F47">
+        <f>INDEX(LINEST(B1:B3,A1:A3),1)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <f>SUM(FREQUENCY(A1:A3,D1:D2))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <f>INDEX(A1:B3,2,2)</f>
         <v>20</v>
       </c>
     </row>
@@ -712,8 +785,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D474A24-3A7D-44AF-A0A5-F07A20834EE0}">
-  <dimension ref="A1:F37"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39C6F16F-B5C2-4C4C-9B79-1AC2A312CA82}">
+  <dimension ref="A1:F49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -968,6 +1041,78 @@
     <row r="37" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F37">
         <f t="array" ref="F37">VLOOKUP(2,A1:B3,2,0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F38">
+        <f t="array" ref="F38">SUMPRODUCT(MAX((C1:C3="x")*B1:B3))</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F39">
+        <f t="array" ref="F39">SUMPRODUCT(LARGE((A1:A3&gt;1)*B1:B3,{1,2}))</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F40">
+        <f t="array" ref="F40">SUMPRODUCT(MAX(LEN(C1:C3)))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F41">
+        <f t="array" ref="F41">LOOKUP(2,1/(A1:A3&gt;1),B1:B3)</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F42">
+        <f t="array" ref="F42">INDEX(B1:B3,MATCH(1,INDEX((A1:A3&gt;1)*(C1:C3="x"),0),0))</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F43">
+        <f t="array" ref="F43">IRR(A1:A3*1-2)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F44">
+        <f t="array" ref="F44">LOOKUP(2,A1:A3,B1:B3)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="45" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F45" t="e">
+        <f t="array" ref="F45">IRR(B1:B3)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="46" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F46">
+        <f t="array" ref="F46">SUM(TREND(B1:B3,A1:A3))</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F47">
+        <f t="array" ref="F47">INDEX(LINEST(B1:B3,A1:A3),1)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="48" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F48">
+        <f t="array" ref="F48">SUM(FREQUENCY(A1:A3,D1:D2))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F49">
+        <f t="array" ref="F49">INDEX(A1:B3,2,2)</f>
         <v>20</v>
       </c>
     </row>
@@ -977,11 +1122,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{257C0EB5-172D-4F73-9C9F-0DD282F22A5B}">
-  <dimension ref="A1:AP3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25496804-CBAB-4FDD-B53B-E7A83DB4B259}">
+  <dimension ref="A1:BB3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A1">
         <v>1</v>
       </c>
@@ -1142,8 +1287,56 @@
         <f>VLOOKUP(2,A1:B3,2,0)</f>
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="AQ1" cm="1">
+        <f t="array" ref="AQ1">SUMPRODUCT(MAX((C1:C3="x")*B1:B3))</f>
+        <v>30</v>
+      </c>
+      <c r="AR1" cm="1">
+        <f t="array" ref="AR1">SUMPRODUCT(LARGE((A1:A3&gt;1)*B1:B3,{1,2}))</f>
+        <v>50</v>
+      </c>
+      <c r="AS1" cm="1">
+        <f t="array" ref="AS1">SUMPRODUCT(MAX(LEN(C1:C3)))</f>
+        <v>1</v>
+      </c>
+      <c r="AT1" cm="1">
+        <f t="array" ref="AT1">LOOKUP(2,1/(A1:A3&gt;1),B1:B3)</f>
+        <v>30</v>
+      </c>
+      <c r="AU1" cm="1">
+        <f t="array" ref="AU1">INDEX(B1:B3,MATCH(1,INDEX((A1:A3&gt;1)*(C1:C3="x"),0),0))</f>
+        <v>30</v>
+      </c>
+      <c r="AV1" s="1" cm="1">
+        <f t="array" ref="AV1">IRR(A1:A3*1-2)</f>
+        <v>0</v>
+      </c>
+      <c r="AW1">
+        <f>LOOKUP(2,A1:A3,B1:B3)</f>
+        <v>20</v>
+      </c>
+      <c r="AX1" s="1" t="e">
+        <f>IRR(B1:B3)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="AY1">
+        <f>SUM(TREND(B1:B3,A1:A3))</f>
+        <v>60</v>
+      </c>
+      <c r="AZ1" cm="1">
+        <f t="array" ref="AZ1">INDEX(LINEST(B1:B3,A1:A3),1)</f>
+        <v>10</v>
+      </c>
+      <c r="BA1">
+        <f>SUM(FREQUENCY(A1:A3,D1:D2))</f>
+        <v>3</v>
+      </c>
+      <c r="BB1">
+        <f>INDEX(A1:B3,2,2)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -1178,7 +1371,7 @@
         <v>y!</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>

</xml_diff>